<commit_message>
feat(track2): refresh iteration-6 submission, pitch deck and explainers
</commit_message>
<xml_diff>
--- a/submissions/track2/iteration-6/agharsallah_track2_methods_form.xlsx
+++ b/submissions/track2/iteration-6/agharsallah_track2_methods_form.xlsx
@@ -679,7 +679,9 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Iteration 6 (Entry 163) unifies our entire Track 2 work across Iterations 1, 2, 4, and 5 into a four-layer, provenance-verified architecture (52 distinct drugs across 13 public databases, served interactively in the React dashboard at /track2, /submissions, and /learn): (1) Five-Instrument Mechanism Characterization &amp; 3D Pocket Plausibility Audit (Entries 129, 147-150, 163): Before naming a medicine, we read the confirmed compound-heterozygous BUB1B genotype (one stop_gained allele + one pseudokinase missense_variant in trans, oracle-confirmed at Rank 1 in entry 083) from five instruments sharing zero data: nine variant-effect models (AlphaMissense top 0.47%, GPN-MSA pair top 0.93%), a Boltz-2 3D fold (local C-alpha RMSD = 0.45 A, entry 147), an all-19,950-substitution ThermoMPNN stability atlas calibrated on published MVA alleles first (placing the child's missense at +1.55 kcal/mol, 87.3rd percentile, inside the 62-residue buried high-confidence pseudokinase core RSA &lt; 0.20 &amp; pLDDT &gt;= 90 where 72.2% of swaps have ddG &gt;= +1.0 kcal/mol -&gt; prior P(unstable)=0.55 vs P(inactive)=0.45, entry 149), a cross-species match of the child's 8 HPO terms against all 76,699 MGI mouse genotypes (selecting the Bub1b^(H/H) hypomorph at top 0.99%, p=0.026, entry 150), and HPO gene ranking (BUB1B #14 of 5,267). Because the missense site is buried inside an occluded non-catalytic pseudokinase core (CDD cd14029, PMID 22561345) rather than a solvent-accessible ligand cavity, distal SIRT2 deacetylation at solvent-exposed Lys668 (NMN, nicotinamide, niacin, PMID 24825348) is biophysically superior to direct orthosteric chaperone docking. (2) Multi-Era Candidate Discovery &amp; Counterfactual Naive-AI Benchmark (Entries 139-160, 163): Combines Iteration 2's 6 directions (D1-D5 + A1/A2) and 5-rung evidence ladder (NAD+/SIRT2 rescues NMN, niacin, nicotinamide PMID 24825348; Rung-5 rhabdomyosarcoma trials simvastatin/lovastatin NCT02390843 + PMID 41249736), Iteration 4's four pre-registered generators tested against a 10,000-draw permutation null (G1 PrimeKG walk, G2 phenotype-twin rescues, G3 919-line PRISM screen sweep, G4 LINCS reversal -&gt; dasatinib sole 2-generator survivor in twin|prism at 99.4th pct aneuploidy, p=0.0096, entry 155), Iteration 5's three routes (Route R1 stop-codon readthrough/NMD context model over 5,837 measured premature stops, R1_score=0.33, &lt;=1.4% WT BubR1, entry 159; Route R2 Gygi-10k HCT116 drug-perturbation proteomics identifying oral gliclazide +1.47 and migalastat +1.44 log2FC BubR1, entry 160; Route R3 42/42 quote-verified literature rows), and a 5-archetype counterfactual benchmark proving why naive bio-AI pipelines fail or harm this child. (3) Per-Child Two-Source Safety, Do-Not Gate &amp; Paediatric PK/PD Translation (Entries 151, 152, 161, 163): K1 excludes Mps1/TTK and Aurora inhibitors (33 of 34 less effective in high-aneuploidy lines, p=0.0096, reproducing PMID 33505028); K2 intersects PharmCAT v3.1.1 on the child's VCF (exposing that variant-only delivery covers 20/1,223 loci = 1.6%) with OnSIDES v3.1.0 drug labels matched to the child's 8 HPO terms (identifying vincristine as the sole drug flagged by both genome CYP3A5 *1/*3 and phenotype HP:0003202 skeletal muscle atrophy); translates all leads to paediatric mg/kg and mg/m^2 regimens, oral liquid/dispersible formulations (e.g. dasatinib PFOS 60-85 mg/m^2/day NCT00777036; simvastatin oral liquid 0.2-0.5 mg/kg/day), muscle/CNS exposure, and monitoring gates. (4) Calibrated Bayesian Decision &amp; Value-of-Information Synthesis (Entries 162, 163): Evaluates all 52 candidates across world-states, sweeps Route-R2 weight w_R2 in [0.05, 1.00], calibrates 1-replicate cell-line proteomics (w_R2=0.25) below multi-animal in vivo Bub1b^(H/H) survival rescues (w_R1=w_R3=1.00), and computes EVPI, EVPPI, and EVSI.</t>
+          <t>Final iteration 6: 52-candidate cross-iteration ledger; mechanism characterization, public-data discovery, per-child safety flags and assumed-weight decision triage. Appendix A and section 6 are generated and checked against canonical TSV/JSON. No clinical efficacy, validated assay accuracy, or patient dosing is claimed.
+Historical methodology context (superseded where audited above):
+Iteration 6 (Entry 163) unifies our entire Track 2 work across Iterations 1, 2, 4, and 5 into a four-layer, provenance-verified architecture (52 distinct drugs across 13 public databases, served interactively in the React dashboard at /track2, /submissions, and /learn): (1) Five-Instrument Mechanism Characterization &amp; 3D Pocket Plausibility Audit (Entries 129, 147-150, 163): Before naming a medicine, we read the confirmed compound-heterozygous BUB1B genotype (one stop_gained allele + one pseudokinase missense_variant in trans, oracle-confirmed at Rank 1 in entry 083) from five instruments sharing zero data: nine variant-effect models (AlphaMissense top 0.47%, GPN-MSA pair top 0.93%), a Boltz-2 3D fold (local C-alpha RMSD = 0.45 A, entry 147), an all-19,950-substitution ThermoMPNN stability atlas calibrated on published MVA alleles first (placing the child's missense at +1.55 kcal/mol, 87.3rd percentile, inside the 62-residue buried high-confidence pseudokinase core RSA &lt; 0.20 &amp; pLDDT &gt;= 90 where 72.2% of swaps have ddG &gt;= +1.0 kcal/mol -&gt; prior P(unstable)=0.55 vs P(inactive)=0.45, entry 149), a cross-species match of the child's 8 HPO terms against all 76,699 MGI mouse genotypes (selecting the Bub1b^(H/H) hypomorph at top 0.99%, p=0.026, entry 150), and HPO gene ranking (BUB1B #14 of 5,267). Because the missense site is buried inside an occluded non-catalytic pseudokinase core (CDD cd14029, PMID 22561345) rather than a solvent-accessible ligand cavity, distal SIRT2 deacetylation at solvent-exposed Lys668 (NMN, nicotinamide, niacin, PMID 24825348) is biophysically superior to direct orthosteric chaperone docking. (2) Multi-Era Candidate Discovery &amp; Counterfactual Naive-AI Benchmark (Entries 139-160, 163): Combines Iteration 2's 6 directions (D1-D5 + A1/A2) and 5-rung evidence ladder (NAD+/SIRT2 rescues NMN, niacin, nicotinamide PMID 24825348; Rung-5 rhabdomyosarcoma trials simvastatin/lovastatin NCT02390843 + PMID 41249736), Iteration 4's four pre-registered generators tested against a 10,000-draw permutation null (G1 PrimeKG walk, G2 phenotype-twin rescues, G3 919-line PRISM screen sweep, G4 LINCS reversal -&gt; dasatinib sole 2-generator survivor in twin|prism at 99.4th pct aneuploidy, p=0.0096, entry 155), Iteration 5's three routes (Route R1 stop-codon readthrough/NMD context model over 5,837 measured premature stops, R1_score=0.33, &lt;=1.4% WT BubR1, entry 159; Route R2 Gygi-10k HCT116 drug-perturbation proteomics identifying oral gliclazide +0.22 and migalastat +0.20 log2FC BubR1, entry 160; Route R3 42/42 quote-verified literature rows), and a 5-archetype counterfactual benchmark proving why naive bio-AI pipelines fail or harm this child. (3) Per-Child Two-Source Safety, Do-Not Gate &amp; Paediatric PK/PD Translation (Entries 151, 152, 161, 163): K1 excludes Mps1/TTK and Aurora inhibitors (33 of 34 less effective in high-aneuploidy lines, p=0.0096, reproducing PMID 33505028); K2 intersects PharmCAT v3.1.1 on the child's VCF (exposing that variant-only delivery covers 20/1,223 loci = 1.6%) with OnSIDES v3.1.0 drug labels matched to the child's 8 HPO terms (identifying vincristine as the sole drug flagged by both genome CYP3A5 *1/*3 and phenotype HP:0003202 skeletal muscle atrophy); translates all leads to paediatric mg/kg and mg/m^2 regimens, oral liquid/dispersible formulations (e.g. dasatinib PFOS 60-85 mg/m^2/day NCT00777036; simvastatin oral liquid 0.2-0.5 mg/kg/day), muscle/CNS exposure, and monitoring gates. (4) Calibrated Bayesian Decision &amp; Value-of-Information Synthesis (Entries 162, 163): Evaluates all 52 candidates across world-states, sweeps Route-R2 weight w_R2 in [0.05, 1.00], calibrates 1-replicate cell-line proteomics (w_R2=0.25) below multi-animal in vivo Bub1b^(H/H) survival rescues (w_R1=w_R3=1.00), and computes EVPI, EVPPI, and EVSI.</t>
         </is>
       </c>
     </row>
@@ -691,7 +693,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Automated computational pipelines gated by pre-registered positive controls and code-enforced checks, combined with bounded, verbatim-verified curation of published experimental parameters. Every generator and route is a deterministic Python tool with a SHA-256 provenance manifest: PrimeKG personalized PageRank (mva.drugs.graph_walk), whole-database MGI semantic matching (tools/phenotype_twin.py), DepMap/PRISM statistical sweeps (tools/screen_sweep.py), SigCom LINCS / iLINCS queries (tools/signature_reversal.py), 10,000-draw Monte Carlo permutation nulls (tools/converge.py), premature-stop readthrough context modeling (src/mva/drugs/stop_context.py), empirical-Bayes and proliferation-regressed proteomics scanning (src/mva/drugs/proteome_perturbation.py), PharmCAT + OnSIDES safety intersection (src/mva/drugs/safety_rerecall.py), 3D pseudokinase core &amp; paediatric PK/PD / counterfactual benchmarking (src/mva/drugs/unified_clinical.py), and calibrated Bayesian Value-of-Information synthesis (src/mva/drugs/unified_synthesis.py). In Route R3 literature mining, an extractor proposed structured rows from 767 Europe PMC papers, but deterministic code verified that every quoted sentence existed verbatim in the cached XML of the cited PMID (42/42 verified, 0 unverified kept). No LLM ranked or selected drugs.</t>
+          <t>Automated computational pipelines gated by pre-registered positive controls and code-enforced checks, combined with bounded, verbatim-verified curation of published experimental parameters. Every generator and route is a deterministic Python tool with a SHA-256 provenance manifest: PrimeKG personalized PageRank (mva.drugs.graph_walk), whole-database MGI semantic matching (tools/phenotype_twin.py), DepMap/PRISM statistical sweeps (tools/screen_sweep.py), SigCom LINCS / iLINCS queries (tools/signature_reversal.py), 10,000-draw Monte Carlo permutation nulls (tools/converge.py), premature-stop readthrough context modeling (src/mva/drugs/stop_context.py), robust residual and proliferation-regressed proteomics scanning (src/mva/drugs/proteome_perturbation.py), PharmCAT + OnSIDES safety intersection (src/mva/drugs/safety_rerecall.py), 3D pseudokinase core &amp; paediatric PK/PD / counterfactual benchmarking (src/mva/drugs/unified_clinical.py), and calibrated Bayesian Value-of-Information synthesis (src/mva/drugs/unified_synthesis.py). In Route R3 literature mining, an extractor proposed structured rows from 767 Europe PMC papers, but deterministic code verified that every quoted sentence existed verbatim in the cached XML of the cited PMID (42/42 verified, 0 unverified kept). No LLM ranked or selected drugs.</t>
         </is>
       </c>
     </row>
@@ -703,7 +705,9 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Manual curation was strictly bounded, recorded in versioned TSVs/modules, and never used to override automated scores: (a) Phenotype-twin interventions (12 rows in entry 150) and Route R3 class analogues (e.g., mapping genetic p16-clearance or tool compounds in Bub1b^(H/H) mice to FDA-approved analogues dasatinib, niacin, nicotinamide, rapamycin) were recorded with verbatim PMIDs (PMID 24825348, 22048312, 27549339) in committed parameter files so any reviewer can inspect them. (b) Published MVA patient allele classes used to calibrate the ThermoMPNN stability atlas (8 alleles: 5 abundance-lowering, 3 stable) were extracted from primary full texts with verbatim quotes (entry 149). (c) The mapping from the proband's 8 HPO terms to MedDRA adverse-event strings (hpo_to_adverse_terms.tsv) was constructed as an explicit lookup table for OnSIDES and openFDA FAERS queries (entry 152). (d) Iteration 2's Rung-5 rhabdomyosarcoma clinical trials (NCT02390843 simvastatin/lovastatin, PMID 41249736) were audited from clinicaltrials.gov and PubMed (entry 144). No drug was manually added to or removed from any automated generator output.</t>
+          <t>Manual curation records literature mechanisms and class analogues, not patient efficacy. Genetic p16-positive-cell clearance is not direct dasatinib treatment evidence. Eight published MVA allele abundance labels (5 low, 3 stable) give ThermoMPNN AUROC .60 with broad interval [.133,1]; the registered test failed. The .55/.45 prior is an assumed triage weight, not established by calibration.
+Historical methodology context (superseded where audited above):
+Manual curation was strictly bounded, recorded in versioned TSVs/modules, and never used to override automated scores: (a) Phenotype-twin interventions (12 rows in entry 150) and Route R3 class analogues (e.g., mapping genetic p16-clearance or tool compounds in Bub1b^(H/H) mice to FDA-approved analogues dasatinib, niacin, nicotinamide, rapamycin) were recorded with verbatim PMIDs (PMID 24825348, 22048312, 27549339) in committed parameter files so any reviewer can inspect them. (b) Published MVA patient allele classes used to calibrate the ThermoMPNN stability atlas (8 alleles: 5 abundance-lowering, 3 stable) were extracted from primary full texts with verbatim quotes (entry 149). (c) The mapping from the proband's 8 HPO terms to MedDRA adverse-event strings (hpo_to_adverse_terms.tsv) was constructed as an explicit lookup table for OnSIDES and openFDA FAERS queries (entry 152). (d) Iteration 2's Rung-5 rhabdomyosarcoma clinical trials (NCT02390843 simvastatin/lovastatin, PMID 41249736) were audited from clinicaltrials.gov and PubMed (entry 144). No drug was manually added to or removed from any automated generator output.</t>
         </is>
       </c>
     </row>
@@ -727,7 +731,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Thirteen public data sources (every downloaded artifact checksummed with URL, SHA-256, and license in .provenance.json manifests): (1) PrimeKG v2.1 (Harvard Dataverse CC0, 129,375 nodes, 8.1M edges, DrugBank-derived drug nodes); (2) ChEMBL v34 REST API, OpenTargets v24.09 GraphQL, and clinicaltrials.gov API v2 (NCT02390843, NCT00492634); (3) Broad Drug Repurposing Hub (6,798 compounds) + PRISM Repurposing primary/secondary screens (578-919 cell lines x 4,518 compounds) + DepMap 24Q2/24Q4 OmicsSomaticMutations, aneuploidy scores, and Model.csv (CC BY 4.0); (4) MGI genotype-phenotype reports (MGI_PhenoGenoMP.rpt, 76,699 mouse genotypes, 402,424 MP assertions), Mammalian Phenotype ontology, HPO (hp.obo + phenotype.hpoa, 12,679 diseases), and Upheno2 / Mouse-Human Mapping Initiative SSSOM (1.10M cross-species equivalences, CC BY 4.0); (5) PharmCAT v3.1.1/v3.4.0 (1,223 CPIC/DPWG allele-defining loci across 19 pharmacogenes) + CPIC API; (6) OnSIDES v3.1.0/v3.1.1 (3,234 FDA drug labels, 4.67M drug-ADE pairs, CC BY 4.0) + openFDA paediatric FAERS; (7) Toledano, Supek &amp; Lehner, Nature Genetics 2024 (PMID 39174735) supplementary table 3 (5,837 measured premature termination codons x 8 readthrough compounds); (8) Gygi-10k / Mitchell et al., Nature Biotechnology 2023 (PMID 36593396 / 38942016, 8,793 perturbations x 9,599 proteins in HCT116) + ProTargetMiner (PMID 31844049); (9) SigCom LINCS &amp; iLINCS L1000 CRISPR-knockout signatures (BUB1B KO across 62 cell lines); (10) AlphaFold DB v6 (AF-O60566-F1-model_v6.pdb), UniProt O60566, Ensembl REST v116, InterPro; (11) ThermoMPNN (MIT) &amp; Boltz-2; (12) AlphaMissense, ESM1b, REVEL, CADD, SpliceAI, GPN-MSA, Evo 2, NT-v2, ESM-C; (13) Europe PMC full-text XML &amp; NCBI PubMed E-utilities.</t>
+          <t>Thirteen public data sources (every downloaded artifact checksummed with URL, SHA-256, and license in .provenance.json manifests): (1) PrimeKG v2.1 (Harvard Dataverse CC0, 129,375 nodes, 8.1M edges, DrugBank-derived drug nodes); (2) ChEMBL v34 REST API, OpenTargets v24.09 GraphQL, and clinicaltrials.gov API v2 (NCT02390843, NCT00492634); (3) Broad Drug Repurposing Hub (6,798 compounds) + PRISM Repurposing primary/secondary screens (578-919 cell lines x 4,518 compounds) + DepMap 24Q2/24Q4 OmicsSomaticMutations, aneuploidy scores, and Model.csv (CC BY 4.0); (4) MGI genotype-phenotype reports (MGI_PhenoGenoMP.rpt, 76,699 mouse genotypes, 402,424 MP assertions), Mammalian Phenotype ontology, HPO (hp.obo + phenotype.hpoa, 12,679 diseases), and Upheno2 / Mouse-Human Mapping Initiative SSSOM (1.10M cross-species equivalences, CC BY 4.0); (5) PharmCAT v3.1.1/v3.4.0 (1,223 CPIC/DPWG allele-defining loci across 19 pharmacogenes) + CPIC API; (6) OnSIDES v3.1.0/v3.1.1 (3,234 FDA drug labels, 4.67M drug-ADE pairs, CC BY 4.0) + openFDA paediatric FAERS; (7) Toledano, Supek &amp; Lehner, Nature Genetics 2024 (PMID 39174735) supplementary table 3 (5,837 measured premature termination codons x 8 readthrough compounds); (8) Gygi-10k / Mitchell et al., Nature Biotechnology 2023 (PMID 36593396 / 36593396, 875 perturbations x 9,599 proteins in HCT116) + ProTargetMiner (PMID 31844049); (9) SigCom LINCS &amp; iLINCS L1000 CRISPR-knockout signatures (BUB1B KO across 62 cell lines); (10) AlphaFold DB v6 (AF-O60566-F1-model_v6.pdb), UniProt O60566, Ensembl REST v116, InterPro; (11) ThermoMPNN (MIT) &amp; Boltz-2; (12) AlphaMissense, ESM1b, REVEL, CADD, SpliceAI, GPN-MSA, Evo 2, NT-v2, ESM-C; (13) Europe PMC full-text XML &amp; NCBI PubMed E-utilities.</t>
         </is>
       </c>
     </row>
@@ -751,7 +755,9 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Loss of function (hypomorphic BubR1 insufficiency) in an oracle-confirmed BUB1B compound heterozygote (one maternal-like stop_gained allele + one paternal-like pseudokinase missense_variant in trans, entry 083). Five independent instruments plus a 3D pseudokinase pocket audit establish the mechanism: (1) Truncating stop_gained allele (entry 159): introduces a UGA premature stop codon (+4 A) in exon 17 of 23, 746 nt upstream of the last exon-exon junction — canonical NMD target lacking the entire C-terminal kinase domain (aa 766-1050) with suboptimal readthrough context (R1_score=0.33; readthrough lifts WT-equivalent BubR1 by at most +1.4 percentage points vs +12.5 for doubling the missense allele). (2) Variant-effect models (entries 129, 148): score the pseudokinase missense in the top 0.47% (AlphaMissense), 2.52% (ESM1b), and 0.93% pair rank (GPN-MSA). (3) All-19,950-substitution ThermoMPNN stability atlas + 3D pseudokinase pocket audit (entries 149, 163): places the child's missense at +1.55 kcal/mol (87.3rd percentile) inside the 62-residue buried high-confidence pseudokinase hydrophobic core (RSA &lt; 0.20, pLDDT &gt;= 90, where 72.2% of swaps have ddG &gt;= +1.0 kcal/mol; Boltz-2 local C-alpha RMSD = 0.45 A), matching the exact profile of published HSP90-dependent, proteasomally degraded MVA alleles (I909T, L1012P, L844F, R727C, R814H, PMID 20516114). Because the missense site is buried in an occluded non-catalytic pseudokinase (CDD cd14029, PMID 22561345), distal Lys668 deacetylation by SIRT2/NAD+ (NMN, nicotinamide, niacin, PMID 24825348) is biophysically favoured over direct active-site chaperone docking, while calibration on 8 published MVA alleles (AUROC=0.60, H083 refuted) establishes the 55%/45% prior (P(unstable)=0.55 vs P(inactive)=0.45). (4) Cross-species phenotype twin (entry 150): independently of the genome, the child's 8 HPO terms select the Bub1b^(H/H) hypomorphic mouse (~10% normal BubR1) in the top 0.99% of 76,699 MGI genotypes (p=0.026). (5) Disrupted pathway: Spindle Assembly Checkpoint (SAC; mitotic checkpoint complex &amp; kinetochore-microtubule attachment via B56-PP2A), causing premature chromatid separation, mosaic variegated aneuploidy, p16^(Ink4a)-mediated cellular senescence, sarcopenia (HP:0003202), growth failure, and embryonal rhabdomyosarcoma (HP:0002859). No evidence supports gain-of-function or dominant-negative activity.</t>
+          <t>BUB1B compound-heterozygous loss of function is the mechanistic hypothesis. Abundance and functional impairment remain unmeasured in this child. Proposed primary patient/parental fibroblast CHX chase at 0,2,4,8h ±MG132; culture and turnaround weeks 1–2, no guaranteed 48h clinical result.
+Historical methodology context (superseded where audited above):
+Loss of function (hypomorphic BubR1 insufficiency) in an oracle-confirmed BUB1B compound heterozygote (one maternal-like stop_gained allele + one paternal-like pseudokinase missense_variant in trans, entry 083). Five independent instruments plus a 3D pseudokinase pocket audit establish the mechanism: (1) Truncating stop_gained allele (entry 159): introduces a UGA premature stop codon (+4 A) in exon 17 of 23, 746 nt upstream of the last exon-exon junction — canonical NMD target lacking the entire C-terminal kinase domain (aa 766-1050) with suboptimal readthrough context (R1_score=0.33; readthrough lifts WT-equivalent BubR1 by at most +1.4 percentage points vs +12.5 for doubling the missense allele). (2) Variant-effect models (entries 129, 148): score the pseudokinase missense in the top 0.47% (AlphaMissense), 2.52% (ESM1b), and 0.93% pair rank (GPN-MSA). (3) All-19,950-substitution ThermoMPNN stability atlas + 3D pseudokinase pocket audit (entries 149, 163): places the child's missense at +1.55 kcal/mol (87.3rd percentile) inside the 62-residue buried high-confidence pseudokinase hydrophobic core (RSA &lt; 0.20, pLDDT &gt;= 90, where 72.2% of swaps have ddG &gt;= +1.0 kcal/mol; Boltz-2 local C-alpha RMSD = 0.45 A), matching the exact profile of published HSP90-dependent, proteasomally degraded MVA alleles (I909T, L1012P, L844F, R727C, R814H, PMID 20516114). Because the missense site is buried in an occluded non-catalytic pseudokinase (CDD cd14029, PMID 22561345), distal Lys668 deacetylation by SIRT2/NAD+ (NMN, nicotinamide, niacin, PMID 24825348) is biophysically favoured over direct active-site chaperone docking, while calibration on 8 published MVA alleles (AUROC=0.60, H083 refuted) establishes the 55%/45% prior (P(unstable)=0.55 vs P(inactive)=0.45). (4) Cross-species phenotype twin (entry 150): independently of the genome, the child's 8 HPO terms select the Bub1b^(H/H) hypomorphic mouse (~10% normal BubR1) in the top 0.99% of 76,699 MGI genotypes (p=0.026). (5) Disrupted pathway: Spindle Assembly Checkpoint (SAC; mitotic checkpoint complex &amp; kinetochore-microtubule attachment via B56-PP2A), causing premature chromatid separation, mosaic variegated aneuploidy, p16^(Ink4a)-mediated cellular senescence, sarcopenia (HP:0003202), growth failure, and embryonal rhabdomyosarcoma (HP:0002859). No evidence supports gain-of-function or dominant-negative activity.</t>
         </is>
       </c>
     </row>
@@ -763,7 +769,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Total compute cost across all Track 2 iterations was $0.015 on Modal T4 GPU (16 GPU-seconds for the 19,950-substitution ThermoMPNN stability atlas in entry 149; plus $14.57 on Modal GPU if counting the shared Track 1 language-model zoo in entry 148) and $0.00 for all drug discovery, proteomics, safety, and Value-of-Information stages on a standard laptop. Wall-clock runtimes: phenotype twin 53 s (entry 150); DepMap/PRISM replication and 613-drug sweep ~4 min (entries 151, 154); PharmCAT + OnSIDES per-child safety &lt;1 min (entries 152, 161); 4-generator convergence + 10,000-draw permutation null 27 s (entry 155); Iteration 5 Routes R1-R4 ~22 min including data downloads and Europe PMC XML retrieval, &lt;15 s from cached tables (entries 159-162); Iteration 6 unified 52-drug synthesis and 20-step calibration sweep &lt;3 s (entry 163); full cross-disease transfer to Bloom syndrome (BLM) 53 min on CPU at $0 (entry 156). Human + AI-assisted engineering effort spanned ~6 days across Step 0 and Iterations 1, 2, 4, 5, and 6 (38 Track 2 methodology entries, 21 pre-registered hypotheses, 25 figures, and unit-tested Python modules).</t>
+          <t>Total GPU cost across all Track 2 iterations was $0.23 on Modal, per the Modal billing report ($0.015 T4 for the 19,950-substitution ThermoMPNN stability atlas in entry 149; $0.17 L4 for the ESM-2 check; $0.04 T4 for the 11-protein abundance calibration; plus $14.57 on Modal GPU if counting the shared Track 1 language-model zoo in entry 148) and $0.00 for all drug discovery, proteomics, safety, and Value-of-Information stages on a standard laptop. Wall-clock runtimes: phenotype twin 53 s (entry 150); DepMap/PRISM replication and 613-drug sweep ~4 min (entries 151, 154); PharmCAT + OnSIDES per-child safety &lt;1 min (entries 152, 161); 4-generator convergence + 10,000-draw permutation null 27 s (entry 155); Iteration 5 Routes R1-R4 ~22 min including data downloads and Europe PMC XML retrieval, &lt;15 s from cached tables (entries 159-162); Iteration 6 unified 52-drug synthesis and 20-step calibration sweep &lt;3 s (entry 163); full cross-disease transfer to Bloom syndrome (BLM) 53 min on CPU at $0 (entry 156). Human + AI-assisted engineering effort spanned ~6 days across Step 0 and Iterations 1, 2, 4, 5, and 6 (38 Track 2 methodology entries, 21 pre-registered hypotheses, 25 figures, and unit-tested Python modules).</t>
         </is>
       </c>
     </row>
@@ -775,10 +781,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Question. Given an oracle-confirmed compound-heterozygous loss of function in BUB1B (one stop_gained and one pseudokinase missense_variant in trans, entry 083) in a child with Mosaic Variegated Aneuploidy 1, skeletal muscle atrophy (HP:0003202), and embryonal rhabdomyosarcoma (HP:0002859), which therapies are scientifically justified, which drugs must be avoided, and what single experiment resolves the remaining uncertainty?
-Approach. Iteration 6 (entry 163) unifies 52 candidates across Iterations 2, 4, and 5 into a four-layer, pre-registered framework. First, five independent instruments read the mechanism: 9 variant-effect models (AlphaMissense top 0.47%), a Boltz-2 fold, an all-19,950-substitution ThermoMPNN stability atlas (+1.55 kcal/mol, 87.3rd percentile, calibrated on published MVA alleles first -&gt; prior P(unstable)=0.55 vs P(inactive)=0.45), and a match of the child's 8 HPO terms against 76,699 MGI mouse genotypes (selecting the Bub1b^(H/H) hypomorph in the top 0.99%, p=0.026). Second, we combine four generators tested against a 10,000-draw permutation null (PrimeKG walk, phenotype-twin rescues, 919-line PRISM sweep, LINCS reversal) with three mechanistic routes: R1 stop-codon readthrough across 5,837 premature stops (R1_score=0.33, contributing &lt;=1.4% WT BubR1), R2 HCT116 drug-perturbation proteomics across 8,793 compounds, and R3 quote-verified Bub1b^(H/H) rescues and rhabdomyosarcoma trials. Third, we apply a two-source per-child safety check (PharmCAT v3.1.1 on the VCF + OnSIDES v3.1.0 HPO-matched drug labels) and a Bayesian Value-of-Information (EVPI/EVPPI/EVSI) model calibrating 1-replicate cell-line proteomics (w_R2=0.25) against in vivo mouse survival rescues (w_R1=w_R3=1.00).
-Results. (1) Next measurement first: across all 20 route-weight steps, EVPI = 0.1800 is invariant, with 100% (EVPPI = 0.1800) on whether the missense allele is unstable vs inactive and 0% (0.0000) on readthrough. A single cycloheximide-chase BubR1 Western blot captures 69.1% of EVPI (EVSI = 0.1245). (2) Pre-blot &amp; if missense_inactive (P=0.45): Dasatinib is the #1 FDA-approved candidate overall (EU=0.2537, u_inactive=0.4000, unflagged), the sole 2-generator survivor (twin|prism, 99.4th pct aneuploidy killing, p=0.0096), and the senolytic analogue of p16-clearance in Bub1b^(H/H) mice (PMID 22048312). (3) If missense_unstable (P=0.55): NMN is #1 overall (u=0.4800, restoring BubR1 via SIRT2 deacetylation in Bub1b^(H/H) mice, PMID 24825348), niacin/nicotinamide are #1 FDA-approved under calibrated R5 (u=0.1920, supported across all 3 iterations), and gliclazide/migalastat are top exploratory R2 proteomic leads (+1.47/+1.44 log2FC BubR1). (4) Presenting rhabdomyosarcoma (D4): Simvastatin/lovastatin (NCT02390843, PMID 41249736), gated on ordering a 5-gene clinical PGx panel (SLCO1B1, ABCG2, CYP2C9, G6PD, UGT1A1) because the variant-only VCF covers 1.6% (20/1,223) of PharmCAT loci. (5) Safety &amp; Do-Not: Vincristine fails both safety arms (CYP3A5 *1/*3 + HP:0003202 muscle atrophy); RYR1 VUS flags anaesthesia risk; 33/34 Mps1/Aurora inhibitors are less effective in aneuploid lines (p=0.0096) and contraindicated.
-Strengths &amp; limitations. Pre-registered hypotheses (8 refutations reported openly), permutation nulls, VOI experimental design, executed transfer to Bloom syndrome ($0, 53 min, Jaccard 0.095). Limitations: 4-generator overlap is at chance level (p=0.263); R2 proteomics is n=1 in HCT116 (control failed, p=0.145); zero candidates have been tested in this child.</t>
+          <t>Research-only synthesis of 52 candidates. Under canonical assumed Se=Sp=.85, P(low)=.535, P(unstable|low)=.8738, P(inactive|normal)=.8226; EVPI=.18, EVSI=.124455 (69.14%). EVPI invariance is structurally .45×.4; zero readthrough information value follows strict dosage feasibility prior zero, distinct from context heuristic .10. External cellular-abundance calibration across 18,825 buried core variants (RSA&lt;.20, pLDDT&gt;=90) in 11 split-disjoint ProteinGym Expression DMS proteins (Modal T4, $0.04): ThermoMPNN median AUROC .7588 (95% CI [.7198,.7783]). For a new protein, P(low abundance | +1.55 kcal/mol) has 95% predictive interval .31–.88 (pooled .6517), which includes .50: Gate B. The .55 prior is kept; the blot decides. Joint sensitivity: 3815/7425 settings (51.38% unweighted grid coverage, not confidence) achieve EVSI&gt;=50% EVPI; EVPI .012–.240, EVSI 0–.2352. No patient-tested therapy or validated assay. FANCA third-disease transfer: partial cached-public MGI/PrimeKG computation, 34 HPO terms, 27.78s; Fanca rank37/76699 symmetric, rank102 Phenodigm; raw top50 graph overlap Jaccard .098901 vs MVA, .041667 vs Bloom. Bounded primary-source audit: raw HCT116 10µM 24h BUB1B log2FC .22 gliclazide and .20 migalastat, one published summary column each. Earlier 1.47/1.44 values are not raw BUB1B log2FC. No independent candidate replication or validated abundance-label expansion found in inspected datasets.</t>
         </is>
       </c>
     </row>

</xml_diff>